<commit_message>
:owl: NMI/CCA p-values check
</commit_message>
<xml_diff>
--- a/data/derived_data/6_NMI_CCA/Dataset_2/CCA_NULL_16S_D2.xlsx
+++ b/data/derived_data/6_NMI_CCA/Dataset_2/CCA_NULL_16S_D2.xlsx
@@ -416,7 +416,7 @@
         <v>1.33158747778634</v>
       </c>
       <c r="E2" t="n">
-        <v>0.274</v>
+        <v>0.247</v>
       </c>
     </row>
     <row r="3">
@@ -433,7 +433,7 @@
         <v>5.08030680642235</v>
       </c>
       <c r="E3" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="4">

</xml_diff>